<commit_message>
Sync planning SharePoint : S22
</commit_message>
<xml_diff>
--- a/Plannings 2026 S22 v2.xlsx
+++ b/Plannings 2026 S22 v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8FC3A8E-B75B-4860-B283-72D6D769F910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{C8FC3A8E-B75B-4860-B283-72D6D769F910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A757388A-A9BB-4520-A4D5-EEA7A8EE8E39}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="147">
   <si>
     <t>Planning des salariés du 25/05/2026 au 31/05/2026</t>
   </si>
@@ -87,9 +87,6 @@
     <t>15:30/18:00</t>
   </si>
   <si>
-    <t>08:45/16:00</t>
-  </si>
-  <si>
     <t>08:45/15:30</t>
   </si>
   <si>
@@ -102,9 +99,6 @@
     <t>18:00/23:30</t>
   </si>
   <si>
-    <t>16:00/20:30</t>
-  </si>
-  <si>
     <t>CASTELLON Pascaline</t>
   </si>
   <si>
@@ -463,6 +457,12 @@
   </si>
   <si>
     <t>EDF // ANNIV // P50M // FINALE LDC</t>
+  </si>
+  <si>
+    <t>08:45/17:30</t>
+  </si>
+  <si>
+    <t>17:30/20:30</t>
   </si>
 </sst>
 </file>
@@ -472,7 +472,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -557,13 +557,6 @@
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Helvetica"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
@@ -913,7 +906,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -989,17 +982,16 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1033,28 +1025,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1066,10 +1058,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -5821,10 +5813,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="110" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00006E000000}"/>
+        <xdr:cNvPr id="114" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000072000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5852,120 +5844,76 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>86</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>86</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="111" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00006F000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>88</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>88</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="112" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000070000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>90</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
       <xdr:row>90</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="113" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000071000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <xdr:cNvPr id="115" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000073000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="116" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000074000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5986,21 +5934,21 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>94</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>94</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="114" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000072000000}"/>
+        <xdr:cNvPr id="117" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000075000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6028,67 +5976,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>92</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>92</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="115" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000073000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>94</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
       <xdr:row>94</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="116" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000074000000}"/>
+        <xdr:cNvPr id="118" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000076000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6116,23 +6020,67 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="119" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000077000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>96</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>96</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="117" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000075000000}"/>
+        <xdr:cNvPr id="120" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000078000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6160,111 +6108,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="118" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000076000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="119" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000077000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>100</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>100</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="120" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000078000000}"/>
+        <xdr:cNvPr id="121" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000079000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6292,103 +6152,59 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="122" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00007A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>101</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
       <xdr:row>101</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="121" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000079000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="114300" cy="114300"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>101</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>101</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="122" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00007A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>103</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>103</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6426,13 +6242,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>101</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>101</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -6690,6 +6506,94 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="130" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12F88D82-923F-4234-B314-82899E464290}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2438400" y="7915275"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="131" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF822338-0B37-44FB-91D1-62DC5599AB43}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7620000" y="12817929"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>101</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -6701,10 +6605,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="130" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12F88D82-923F-4234-B314-82899E464290}"/>
+        <xdr:cNvPr id="134" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23D41503-ED1C-4271-8F96-1E3E49211F78}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6720,7 +6624,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2438400" y="7915275"/>
+          <a:off x="7620000" y="16287750"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -6734,21 +6638,21 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>66</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="131" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF822338-0B37-44FB-91D1-62DC5599AB43}"/>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="135" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4578624C-EA9F-4D3E-A3FA-A867441F5EF6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6764,35 +6668,167 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7620000" y="12817929"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
+          <a:off x="11430000" y="12817929"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="136" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B174561-FC72-4C49-9743-28ED5947FACC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19050000" y="5061857"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="41" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{585254C2-0F2D-4FC0-BAC6-0CB9A1A9BC7E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22860000" y="16764000"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="61" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFB7C3B3-963F-467B-8547-263381171AF5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22860000" y="17145000"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>103</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
       <xdr:row>103</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="134" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23D41503-ED1C-4271-8F96-1E3E49211F78}"/>
+        <xdr:cNvPr id="132" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{84B49583-7442-4A02-A9B0-DC07E854F8CB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6808,95 +6844,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7620000" y="16287750"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>101</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>101</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="135" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4578624C-EA9F-4D3E-A3FA-A867441F5EF6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11430000" y="12817929"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="136" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3B174561-FC72-4C49-9743-28ED5947FACC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19050000" y="5061857"/>
+          <a:off x="22860000" y="17526000"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7285,48 +7233,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="56" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="E3" s="12" t="s">
+      <c r="G3" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="F3" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>146</v>
-      </c>
       <c r="H3" s="12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7356,7 +7304,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="57" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="13"/>
@@ -7364,25 +7312,25 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="31" t="s">
         <v>12</v>
       </c>
       <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="59"/>
+      <c r="A6" s="58"/>
       <c r="B6" s="16"/>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
-      <c r="G6" s="41" t="s">
+      <c r="G6" s="40" t="s">
         <v>13</v>
       </c>
       <c r="H6" s="18"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="57" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="13"/>
@@ -7396,7 +7344,7 @@
       <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="59"/>
+      <c r="A8" s="58"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
       <c r="D8" s="17" t="s">
@@ -7408,7 +7356,7 @@
       <c r="H8" s="18"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="57" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="14"/>
@@ -7430,7 +7378,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="60"/>
+      <c r="A10" s="59"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
         <v>18</v>
@@ -7443,46 +7391,46 @@
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="H10" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="19" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="60"/>
+      <c r="A11" s="59"/>
       <c r="C11" s="1"/>
       <c r="D11" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="54" t="s">
-        <v>141</v>
+        <v>22</v>
+      </c>
+      <c r="E11" s="53" t="s">
+        <v>139</v>
       </c>
       <c r="F11" s="1"/>
-      <c r="G11" s="55" t="s">
-        <v>142</v>
+      <c r="G11" s="54" t="s">
+        <v>140</v>
       </c>
       <c r="H11" s="19"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="59"/>
+      <c r="A12" s="58"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="30" t="s">
+      <c r="F12" s="17"/>
+      <c r="G12" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="H12" s="18"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="57" t="s">
         <v>25</v>
-      </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="18"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="58" t="s">
-        <v>27</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="14"/>
@@ -7495,24 +7443,24 @@
       <c r="H13" s="15"/>
     </row>
     <row r="14" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="59"/>
+      <c r="A14" s="58"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
       <c r="H14" s="18"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="58" t="s">
-        <v>29</v>
+      <c r="A15" s="57" t="s">
+        <v>27</v>
       </c>
       <c r="B15" s="13"/>
       <c r="C15" s="24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
@@ -7521,10 +7469,10 @@
       <c r="H15" s="15"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="60"/>
+      <c r="A16" s="59"/>
       <c r="B16" s="1"/>
       <c r="C16" s="25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -7533,7 +7481,7 @@
       <c r="H16" s="19"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="60"/>
+      <c r="A17" s="59"/>
       <c r="B17" s="1"/>
       <c r="C17" s="2" t="s">
         <v>15</v>
@@ -7545,10 +7493,10 @@
       <c r="H17" s="19"/>
     </row>
     <row r="18" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="59"/>
+      <c r="A18" s="58"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
@@ -7557,15 +7505,15 @@
       <c r="H18" s="18"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="58" t="s">
-        <v>33</v>
+      <c r="A19" s="57" t="s">
+        <v>31</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="39" t="s">
-        <v>34</v>
+      <c r="D19" s="38" t="s">
+        <v>32</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>15</v>
@@ -7577,25 +7525,25 @@
       <c r="H19" s="15"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="60"/>
+      <c r="A20" s="59"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="40" t="s">
+      <c r="F20" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="G20" s="1"/>
       <c r="H20" s="19"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="60"/>
+      <c r="A21" s="59"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="2" t="s">
@@ -7607,11 +7555,11 @@
       <c r="H21" s="19"/>
     </row>
     <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="61"/>
+      <c r="A22" s="60"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -7619,8 +7567,8 @@
       <c r="H22" s="19"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="58" t="s">
-        <v>40</v>
+      <c r="A23" s="57" t="s">
+        <v>38</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="14" t="s">
@@ -7637,184 +7585,184 @@
       <c r="H23" s="15"/>
     </row>
     <row r="24" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="59"/>
+      <c r="A24" s="58"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D24" s="17"/>
       <c r="E24" s="17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F24" s="17"/>
       <c r="G24" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H24" s="18"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="57" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="H24" s="18"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="58" t="s">
+      <c r="C25" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="14"/>
+      <c r="F25" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="G25" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="H25" s="15"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="59"/>
+      <c r="B26" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="1"/>
+      <c r="F26" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" s="19"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="59"/>
+      <c r="B27" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B25" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="E25" s="14"/>
-      <c r="F25" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="G25" s="36" t="s">
+      <c r="C27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="G27" s="36"/>
+      <c r="H27" s="19"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="59"/>
+      <c r="B28" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H25" s="15"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="60"/>
-      <c r="B26" s="33" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="33" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="33" t="s">
-        <v>49</v>
-      </c>
-      <c r="G26" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="H26" s="19"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="60"/>
-      <c r="B27" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="E27" s="1"/>
-      <c r="F27" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="G27" s="37"/>
-      <c r="H27" s="19"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="60"/>
-      <c r="B28" s="1" t="s">
+      <c r="D28" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="E28" s="1"/>
+      <c r="F28" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="G28" s="36"/>
+      <c r="H28" s="19"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="59"/>
+      <c r="B29" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E28" s="1"/>
-      <c r="F28" s="37" t="s">
+      <c r="E29" s="1"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="19"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="59"/>
+      <c r="B30" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="G28" s="37"/>
-      <c r="H28" s="19"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="60"/>
-      <c r="B29" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="C29" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="C30" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="E29" s="1"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="37"/>
-      <c r="H29" s="19"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="60"/>
-      <c r="B30" s="33" t="s">
+      <c r="D30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C30" s="33" t="s">
+      <c r="E30" s="1"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="19"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="59"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="E31" s="1"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="36"/>
+      <c r="H31" s="19"/>
+    </row>
+    <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="59"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="E32" s="1"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="19"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="57" t="s">
         <v>59</v>
-      </c>
-      <c r="E30" s="1"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="37"/>
-      <c r="H30" s="19"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="60"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="E31" s="1"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="19"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="60"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="33"/>
-      <c r="D32" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="E32" s="1"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="19"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="58" t="s">
-        <v>61</v>
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
       <c r="E33" s="14"/>
       <c r="F33" s="14"/>
-      <c r="G33" s="32" t="s">
+      <c r="G33" s="31" t="s">
         <v>12</v>
       </c>
       <c r="H33" s="15"/>
     </row>
     <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="59"/>
+      <c r="A34" s="58"/>
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
       <c r="E34" s="17"/>
       <c r="F34" s="17"/>
-      <c r="G34" s="41" t="s">
+      <c r="G34" s="40" t="s">
         <v>13</v>
       </c>
       <c r="H34" s="18"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="58" t="s">
-        <v>62</v>
+      <c r="A35" s="57" t="s">
+        <v>60</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>15</v>
@@ -7828,39 +7776,39 @@
         <v>15</v>
       </c>
       <c r="G35" s="14"/>
-      <c r="H35" s="43" t="s">
-        <v>63</v>
+      <c r="H35" s="42" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="60"/>
+      <c r="A36" s="59"/>
       <c r="B36" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G36" s="1"/>
+      <c r="H36" s="43" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="59"/>
+      <c r="B37" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="44" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="60"/>
-      <c r="B37" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="1"/>
-      <c r="D37" s="34" t="s">
-        <v>68</v>
-      </c>
       <c r="E37" s="1"/>
-      <c r="F37" s="34" t="s">
+      <c r="F37" s="33" t="s">
         <v>12</v>
       </c>
       <c r="G37" s="1"/>
@@ -7869,25 +7817,25 @@
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="60"/>
-      <c r="B38" s="33" t="s">
-        <v>69</v>
+      <c r="A38" s="59"/>
+      <c r="B38" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="C38" s="1"/>
-      <c r="D38" s="33" t="s">
-        <v>70</v>
+      <c r="D38" s="32" t="s">
+        <v>68</v>
       </c>
       <c r="E38" s="1"/>
-      <c r="F38" s="33" t="s">
-        <v>69</v>
+      <c r="F38" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="19" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="60"/>
+      <c r="A39" s="59"/>
       <c r="B39" s="2" t="s">
         <v>15</v>
       </c>
@@ -7896,50 +7844,50 @@
         <v>15</v>
       </c>
       <c r="E39" s="1"/>
-      <c r="F39" s="33"/>
+      <c r="F39" s="32"/>
       <c r="G39" s="1"/>
       <c r="H39" s="19"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="60"/>
+      <c r="A40" s="59"/>
       <c r="B40" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E40" s="1"/>
-      <c r="F40" s="33"/>
+      <c r="F40" s="32"/>
       <c r="G40" s="1"/>
       <c r="H40" s="19"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="60"/>
+      <c r="A41" s="59"/>
       <c r="C41" s="1"/>
-      <c r="D41" s="34" t="s">
-        <v>68</v>
+      <c r="D41" s="33" t="s">
+        <v>66</v>
       </c>
       <c r="E41" s="1"/>
-      <c r="F41" s="33"/>
+      <c r="F41" s="32"/>
       <c r="G41" s="1"/>
       <c r="H41" s="19"/>
     </row>
     <row r="42" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="59"/>
+      <c r="A42" s="58"/>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
-      <c r="D42" s="41" t="s">
-        <v>73</v>
+      <c r="D42" s="40" t="s">
+        <v>71</v>
       </c>
       <c r="E42" s="17"/>
-      <c r="F42" s="41"/>
+      <c r="F42" s="40"/>
       <c r="G42" s="17"/>
       <c r="H42" s="18"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="58" t="s">
-        <v>74</v>
+      <c r="A43" s="57" t="s">
+        <v>72</v>
       </c>
       <c r="B43" s="13"/>
       <c r="C43" s="14"/>
@@ -7952,12 +7900,12 @@
       <c r="H43" s="15"/>
     </row>
     <row r="44" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="59"/>
+      <c r="A44" s="58"/>
       <c r="B44" s="17"/>
       <c r="C44" s="17"/>
       <c r="D44" s="17"/>
       <c r="E44" s="17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F44" s="17"/>
       <c r="G44" s="17"/>
@@ -7965,19 +7913,19 @@
     </row>
     <row r="45" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="B45" s="63"/>
-      <c r="C45" s="64"/>
-      <c r="D45" s="64"/>
-      <c r="E45" s="64"/>
-      <c r="F45" s="64"/>
-      <c r="G45" s="64"/>
-      <c r="H45" s="65"/>
+        <v>74</v>
+      </c>
+      <c r="B45" s="62"/>
+      <c r="C45" s="63"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="63"/>
+      <c r="F45" s="63"/>
+      <c r="G45" s="63"/>
+      <c r="H45" s="64"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="58" t="s">
-        <v>77</v>
+      <c r="A46" s="57" t="s">
+        <v>75</v>
       </c>
       <c r="B46" s="13"/>
       <c r="C46" s="14"/>
@@ -7990,7 +7938,7 @@
       </c>
     </row>
     <row r="47" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="59"/>
+      <c r="A47" s="58"/>
       <c r="B47" s="17"/>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -7998,12 +7946,12 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
       <c r="H47" s="18" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="58" t="s">
-        <v>79</v>
+      <c r="A48" s="57" t="s">
+        <v>77</v>
       </c>
       <c r="B48" s="13"/>
       <c r="C48" s="14"/>
@@ -8011,81 +7959,81 @@
       <c r="E48" s="14"/>
       <c r="F48" s="14"/>
       <c r="G48" s="14"/>
-      <c r="H48" s="43" t="s">
-        <v>63</v>
+      <c r="H48" s="42" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="60"/>
+      <c r="A49" s="59"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
-      <c r="H49" s="44" t="s">
-        <v>49</v>
+      <c r="H49" s="43" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="60"/>
+      <c r="A50" s="59"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
-      <c r="H50" s="51" t="s">
-        <v>30</v>
+      <c r="H50" s="50" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="59"/>
+      <c r="A51" s="58"/>
       <c r="B51" s="17"/>
       <c r="C51" s="17"/>
       <c r="D51" s="17"/>
       <c r="E51" s="17"/>
       <c r="F51" s="17"/>
       <c r="G51" s="17"/>
-      <c r="H51" s="53" t="s">
-        <v>80</v>
+      <c r="H51" s="52" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="58" t="s">
-        <v>81</v>
+      <c r="A52" s="57" t="s">
+        <v>79</v>
       </c>
       <c r="B52" s="13"/>
       <c r="C52" s="14"/>
-      <c r="D52" s="32" t="s">
+      <c r="D52" s="31" t="s">
         <v>12</v>
       </c>
       <c r="E52" s="14"/>
       <c r="F52" s="24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G52" s="14"/>
       <c r="H52" s="15"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="60"/>
+      <c r="A53" s="59"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
-      <c r="D53" s="33" t="s">
-        <v>49</v>
+      <c r="D53" s="32" t="s">
+        <v>47</v>
       </c>
       <c r="E53" s="1"/>
       <c r="F53" s="25" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" s="19"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="60"/>
+      <c r="A54" s="59"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
-      <c r="D54" s="33"/>
+      <c r="D54" s="32"/>
       <c r="E54" s="1"/>
       <c r="F54" s="2" t="s">
         <v>12</v>
@@ -8094,169 +8042,169 @@
       <c r="H54" s="19"/>
     </row>
     <row r="55" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="59"/>
+      <c r="A55" s="58"/>
       <c r="B55" s="17"/>
       <c r="C55" s="17"/>
-      <c r="D55" s="41"/>
-      <c r="E55" s="42"/>
+      <c r="D55" s="40"/>
+      <c r="E55" s="41"/>
       <c r="F55" s="17" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G55" s="17"/>
       <c r="H55" s="18"/>
     </row>
     <row r="56" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="B56" s="66"/>
-      <c r="C56" s="67"/>
-      <c r="D56" s="67"/>
-      <c r="E56" s="67"/>
-      <c r="F56" s="67"/>
-      <c r="G56" s="67"/>
-      <c r="H56" s="68"/>
+        <v>81</v>
+      </c>
+      <c r="B56" s="65"/>
+      <c r="C56" s="66"/>
+      <c r="D56" s="66"/>
+      <c r="E56" s="66"/>
+      <c r="F56" s="66"/>
+      <c r="G56" s="66"/>
+      <c r="H56" s="67"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="58" t="s">
-        <v>84</v>
+      <c r="A57" s="57" t="s">
+        <v>82</v>
       </c>
       <c r="B57" s="13"/>
       <c r="C57" s="14"/>
       <c r="D57" s="14"/>
       <c r="E57" s="14"/>
       <c r="F57" s="14"/>
-      <c r="G57" s="45" t="s">
-        <v>63</v>
+      <c r="G57" s="44" t="s">
+        <v>61</v>
       </c>
       <c r="H57" s="15" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="60"/>
+      <c r="A58" s="59"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
-      <c r="G58" s="46" t="s">
-        <v>85</v>
+      <c r="G58" s="45" t="s">
+        <v>83</v>
       </c>
       <c r="H58" s="19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="60"/>
+      <c r="A59" s="59"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
-      <c r="G59" s="47" t="s">
-        <v>87</v>
-      </c>
-      <c r="H59" s="49" t="s">
-        <v>63</v>
+      <c r="G59" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="H59" s="48" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="60"/>
+      <c r="A60" s="59"/>
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
       <c r="F60" s="1"/>
-      <c r="G60" s="46" t="s">
-        <v>88</v>
-      </c>
-      <c r="H60" s="44" t="s">
-        <v>89</v>
+      <c r="G60" s="45" t="s">
+        <v>86</v>
+      </c>
+      <c r="H60" s="43" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="60"/>
+      <c r="A61" s="59"/>
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
       <c r="F61" s="1"/>
-      <c r="G61" s="46"/>
+      <c r="G61" s="45"/>
       <c r="H61" s="20" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="60"/>
+      <c r="A62" s="59"/>
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
       <c r="F62" s="1"/>
-      <c r="G62" s="46"/>
+      <c r="G62" s="45"/>
       <c r="H62" s="19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A63" s="60"/>
+      <c r="A63" s="59"/>
       <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
       <c r="E63" s="1"/>
       <c r="F63" s="1"/>
-      <c r="G63" s="46"/>
-      <c r="H63" s="49" t="s">
-        <v>63</v>
+      <c r="G63" s="45"/>
+      <c r="H63" s="48" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="60"/>
+      <c r="A64" s="59"/>
       <c r="B64" s="1"/>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
       <c r="E64" s="1"/>
       <c r="F64" s="1"/>
-      <c r="G64" s="46"/>
-      <c r="H64" s="44" t="s">
-        <v>91</v>
+      <c r="G64" s="45"/>
+      <c r="H64" s="43" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="60"/>
+      <c r="A65" s="59"/>
       <c r="B65" s="1"/>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1"/>
-      <c r="G65" s="46"/>
-      <c r="H65" s="51" t="s">
-        <v>30</v>
+      <c r="G65" s="45"/>
+      <c r="H65" s="50" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="59"/>
+      <c r="A66" s="58"/>
       <c r="B66" s="17"/>
       <c r="C66" s="17"/>
       <c r="D66" s="17"/>
       <c r="E66" s="17"/>
       <c r="F66" s="17"/>
-      <c r="G66" s="48"/>
-      <c r="H66" s="53" t="s">
-        <v>52</v>
+      <c r="G66" s="47"/>
+      <c r="H66" s="52" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" s="58" t="s">
-        <v>92</v>
+      <c r="A67" s="57" t="s">
+        <v>90</v>
       </c>
       <c r="B67" s="13"/>
-      <c r="C67" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="D67" s="31" t="s">
-        <v>93</v>
+      <c r="C67" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="D67" s="30" t="s">
+        <v>91</v>
       </c>
       <c r="E67" s="14"/>
       <c r="F67" s="14"/>
@@ -8264,13 +8212,13 @@
       <c r="H67" s="15"/>
     </row>
     <row r="68" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="59"/>
+      <c r="A68" s="58"/>
       <c r="B68" s="17"/>
-      <c r="C68" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="D68" s="30" t="s">
-        <v>94</v>
+      <c r="C68" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="D68" s="29" t="s">
+        <v>92</v>
       </c>
       <c r="E68" s="17"/>
       <c r="F68" s="17"/>
@@ -8278,13 +8226,13 @@
       <c r="H68" s="18"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" s="58" t="s">
-        <v>95</v>
+      <c r="A69" s="57" t="s">
+        <v>93</v>
       </c>
       <c r="B69" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C69" s="32" t="s">
+      <c r="C69" s="31" t="s">
         <v>12</v>
       </c>
       <c r="D69" s="14"/>
@@ -8294,12 +8242,12 @@
       <c r="H69" s="15"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="60"/>
+      <c r="A70" s="59"/>
       <c r="B70" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C70" s="33" t="s">
-        <v>69</v>
+        <v>94</v>
+      </c>
+      <c r="C70" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
@@ -8308,9 +8256,9 @@
       <c r="H70" s="19"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A71" s="60"/>
+      <c r="A71" s="59"/>
       <c r="C71" s="27" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
@@ -8319,10 +8267,10 @@
       <c r="H71" s="19"/>
     </row>
     <row r="72" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="59"/>
+      <c r="A72" s="58"/>
       <c r="B72" s="17"/>
-      <c r="C72" s="30" t="s">
-        <v>97</v>
+      <c r="C72" s="29" t="s">
+        <v>95</v>
       </c>
       <c r="D72" s="17"/>
       <c r="E72" s="17"/>
@@ -8331,66 +8279,66 @@
       <c r="H72" s="18"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A73" s="58" t="s">
-        <v>98</v>
+      <c r="A73" s="57" t="s">
+        <v>96</v>
       </c>
       <c r="B73" s="13"/>
       <c r="C73" s="24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D73" s="14"/>
       <c r="E73" s="14"/>
-      <c r="F73" s="32" t="s">
+      <c r="F73" s="31" t="s">
         <v>12</v>
       </c>
       <c r="G73" s="14"/>
-      <c r="H73" s="43" t="s">
-        <v>63</v>
+      <c r="H73" s="42" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" s="60"/>
+      <c r="A74" s="59"/>
       <c r="B74" s="1"/>
       <c r="C74" s="25" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
-      <c r="F74" s="33" t="s">
-        <v>69</v>
+      <c r="F74" s="32" t="s">
+        <v>67</v>
       </c>
       <c r="G74" s="1"/>
-      <c r="H74" s="44" t="s">
-        <v>99</v>
+      <c r="H74" s="43" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" s="60"/>
+      <c r="A75" s="59"/>
       <c r="B75" s="1"/>
-      <c r="C75" s="34" t="s">
+      <c r="C75" s="33" t="s">
         <v>12</v>
       </c>
       <c r="D75" s="1"/>
       <c r="E75" s="1"/>
-      <c r="F75" s="33"/>
+      <c r="F75" s="32"/>
       <c r="G75" s="1"/>
-      <c r="H75" s="44"/>
+      <c r="H75" s="43"/>
     </row>
     <row r="76" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="59"/>
+      <c r="A76" s="58"/>
       <c r="B76" s="17"/>
-      <c r="C76" s="41" t="s">
-        <v>69</v>
+      <c r="C76" s="40" t="s">
+        <v>67</v>
       </c>
       <c r="D76" s="17"/>
       <c r="E76" s="17"/>
-      <c r="F76" s="41"/>
+      <c r="F76" s="40"/>
       <c r="G76" s="17"/>
-      <c r="H76" s="50"/>
+      <c r="H76" s="49"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A77" s="58" t="s">
-        <v>100</v>
+      <c r="A77" s="57" t="s">
+        <v>98</v>
       </c>
       <c r="B77" s="14" t="s">
         <v>15</v>
@@ -8413,64 +8361,64 @@
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A78" s="60"/>
+      <c r="A78" s="59"/>
       <c r="B78" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="E78" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D78" s="1" t="s">
+      <c r="F78" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="G78" s="1"/>
       <c r="H78" s="19" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A79" s="60"/>
+      <c r="A79" s="59"/>
       <c r="C79" s="26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D79" s="26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E79" s="1"/>
       <c r="F79" s="26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G79" s="1"/>
-      <c r="H79" s="51" t="s">
-        <v>30</v>
+      <c r="H79" s="50" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A80" s="60"/>
+      <c r="A80" s="59"/>
       <c r="B80" s="1"/>
       <c r="C80" s="25" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D80" s="25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E80" s="1"/>
       <c r="F80" s="25" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G80" s="1"/>
-      <c r="H80" s="52" t="s">
-        <v>109</v>
+      <c r="H80" s="51" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A81" s="60"/>
+      <c r="A81" s="59"/>
       <c r="B81" s="1"/>
       <c r="C81" s="2" t="s">
         <v>15</v>
@@ -8483,50 +8431,50 @@
         <v>15</v>
       </c>
       <c r="G81" s="1"/>
-      <c r="H81" s="52"/>
+      <c r="H81" s="51"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A82" s="60"/>
+      <c r="A82" s="59"/>
       <c r="B82" s="1"/>
       <c r="C82" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E82" s="1"/>
       <c r="F82" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G82" s="1"/>
-      <c r="H82" s="52"/>
+      <c r="H82" s="51"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A83" s="60"/>
+      <c r="A83" s="59"/>
       <c r="B83" s="1"/>
       <c r="C83" s="26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D83" s="1"/>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
-      <c r="H83" s="52"/>
+      <c r="H83" s="51"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A84" s="60"/>
+      <c r="A84" s="59"/>
       <c r="B84" s="1"/>
       <c r="C84" s="25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D84" s="1"/>
       <c r="E84" s="1"/>
       <c r="F84" s="1"/>
       <c r="G84" s="1"/>
-      <c r="H84" s="52"/>
+      <c r="H84" s="51"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A85" s="60"/>
+      <c r="A85" s="59"/>
       <c r="B85" s="1"/>
       <c r="C85" s="2" t="s">
         <v>15</v>
@@ -8535,23 +8483,23 @@
       <c r="E85" s="1"/>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
-      <c r="H85" s="52"/>
+      <c r="H85" s="51"/>
     </row>
     <row r="86" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="59"/>
+      <c r="A86" s="58"/>
       <c r="B86" s="17"/>
       <c r="C86" s="17" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D86" s="17"/>
       <c r="E86" s="17"/>
       <c r="F86" s="17"/>
       <c r="G86" s="17"/>
-      <c r="H86" s="53"/>
+      <c r="H86" s="52"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A87" s="58" t="s">
-        <v>114</v>
+      <c r="A87" s="57" t="s">
+        <v>112</v>
       </c>
       <c r="B87" s="14" t="s">
         <v>15</v>
@@ -8560,220 +8508,216 @@
       <c r="D87" s="14"/>
       <c r="E87" s="14"/>
       <c r="F87" s="14"/>
-      <c r="G87" s="14" t="s">
-        <v>15</v>
-      </c>
+      <c r="G87" s="14"/>
       <c r="H87" s="15"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A88" s="60"/>
+      <c r="A88" s="59"/>
       <c r="B88" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C88" s="1"/>
       <c r="D88" s="1"/>
       <c r="E88" s="1"/>
       <c r="F88" s="1"/>
-      <c r="G88" s="1" t="s">
-        <v>116</v>
-      </c>
+      <c r="G88" s="1"/>
       <c r="H88" s="19"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A89" s="60"/>
+      <c r="A89" s="59"/>
       <c r="B89" s="27" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C89" s="1"/>
       <c r="D89" s="1"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
-      <c r="G89" s="47" t="s">
-        <v>63</v>
-      </c>
+      <c r="G89" s="1"/>
       <c r="H89" s="19"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A90" s="60"/>
+    <row r="90" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="59"/>
       <c r="B90" s="28" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
-      <c r="G90" s="46" t="s">
-        <v>99</v>
-      </c>
+      <c r="G90" s="1"/>
       <c r="H90" s="19"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A91" s="60"/>
-      <c r="B91" s="29"/>
-      <c r="C91" s="1"/>
-      <c r="D91" s="1"/>
-      <c r="E91" s="1"/>
-      <c r="F91" s="1"/>
-      <c r="G91" s="2" t="s">
+      <c r="A91" s="57" t="s">
+        <v>116</v>
+      </c>
+      <c r="B91" s="13"/>
+      <c r="C91" s="14"/>
+      <c r="D91" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E91" s="14"/>
+      <c r="F91" s="14"/>
+      <c r="G91" s="14"/>
+      <c r="H91" s="15"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="59"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="19"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="59"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
+      <c r="D93" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="19"/>
+    </row>
+    <row r="94" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="58"/>
+      <c r="B94" s="17"/>
+      <c r="C94" s="17"/>
+      <c r="D94" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="E94" s="17"/>
+      <c r="F94" s="17"/>
+      <c r="G94" s="17"/>
+      <c r="H94" s="18"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="57" t="s">
+        <v>117</v>
+      </c>
+      <c r="B95" s="13"/>
+      <c r="C95" s="14"/>
+      <c r="D95" s="14"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="14"/>
+      <c r="G95" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="H95" s="55"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="59"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="H96" s="19"/>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A97" s="59"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="F97" s="1"/>
+      <c r="G97" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="H97" s="19"/>
+    </row>
+    <row r="98" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="58"/>
+      <c r="B98" s="17"/>
+      <c r="C98" s="17"/>
+      <c r="D98" s="17"/>
+      <c r="E98" s="17"/>
+      <c r="F98" s="17"/>
+      <c r="G98" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="H98" s="18"/>
+    </row>
+    <row r="99" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B99" s="62"/>
+      <c r="C99" s="63"/>
+      <c r="D99" s="63"/>
+      <c r="E99" s="63"/>
+      <c r="F99" s="63"/>
+      <c r="G99" s="63"/>
+      <c r="H99" s="64"/>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A100" s="57" t="s">
+        <v>120</v>
+      </c>
+      <c r="B100" s="13"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="30" t="s">
+        <v>91</v>
+      </c>
+      <c r="E100" s="14"/>
+      <c r="F100" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="G100" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H91" s="19"/>
-    </row>
-    <row r="92" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="59"/>
-      <c r="B92" s="30"/>
-      <c r="C92" s="17"/>
-      <c r="D92" s="17"/>
-      <c r="E92" s="17"/>
-      <c r="F92" s="17"/>
-      <c r="G92" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="H92" s="18"/>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A93" s="58" t="s">
-        <v>118</v>
-      </c>
-      <c r="B93" s="13"/>
-      <c r="C93" s="14"/>
-      <c r="D93" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="E93" s="14"/>
-      <c r="F93" s="14"/>
-      <c r="G93" s="14"/>
-      <c r="H93" s="15"/>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A94" s="60"/>
-      <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
-      <c r="D94" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="E94" s="1"/>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
-      <c r="H94" s="19"/>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A95" s="60"/>
-      <c r="B95" s="1"/>
-      <c r="C95" s="1"/>
-      <c r="D95" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="E95" s="1"/>
-      <c r="F95" s="1"/>
-      <c r="G95" s="1"/>
-      <c r="H95" s="19"/>
-    </row>
-    <row r="96" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="59"/>
-      <c r="B96" s="17"/>
-      <c r="C96" s="17"/>
-      <c r="D96" s="41" t="s">
-        <v>49</v>
-      </c>
-      <c r="E96" s="17"/>
-      <c r="F96" s="17"/>
-      <c r="G96" s="17"/>
-      <c r="H96" s="18"/>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A97" s="58" t="s">
-        <v>119</v>
-      </c>
-      <c r="B97" s="13"/>
-      <c r="C97" s="14"/>
-      <c r="D97" s="14"/>
-      <c r="E97" s="14"/>
-      <c r="F97" s="14"/>
-      <c r="G97" s="32" t="s">
-        <v>12</v>
-      </c>
-      <c r="H97" s="56"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A98" s="60"/>
-      <c r="B98" s="1"/>
-      <c r="C98" s="1"/>
-      <c r="D98" s="1"/>
-      <c r="E98" s="1"/>
-      <c r="F98" s="1"/>
-      <c r="G98" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="H98" s="19"/>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A99" s="60"/>
-      <c r="B99" s="1"/>
-      <c r="C99" s="1"/>
-      <c r="D99" s="1"/>
-      <c r="E99" s="1"/>
-      <c r="F99" s="1"/>
-      <c r="G99" s="34" t="s">
-        <v>12</v>
-      </c>
-      <c r="H99" s="19"/>
-    </row>
-    <row r="100" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="59"/>
-      <c r="B100" s="17"/>
-      <c r="C100" s="17"/>
-      <c r="D100" s="17"/>
-      <c r="E100" s="17"/>
-      <c r="F100" s="17"/>
-      <c r="G100" s="41" t="s">
-        <v>120</v>
-      </c>
-      <c r="H100" s="18"/>
-    </row>
-    <row r="101" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="B101" s="63"/>
-      <c r="C101" s="64"/>
-      <c r="D101" s="64"/>
-      <c r="E101" s="64"/>
-      <c r="F101" s="64"/>
-      <c r="G101" s="64"/>
-      <c r="H101" s="65"/>
+      <c r="H100" s="15"/>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A101" s="59"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+      <c r="D101" s="28" t="s">
+        <v>95</v>
+      </c>
+      <c r="E101" s="1"/>
+      <c r="F101" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="H101" s="19"/>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A102" s="58" t="s">
-        <v>122</v>
-      </c>
-      <c r="B102" s="13"/>
-      <c r="C102" s="14"/>
-      <c r="D102" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="E102" s="14"/>
-      <c r="F102" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="G102" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="H102" s="15"/>
+      <c r="A102" s="59"/>
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+      <c r="D102" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E102" s="1"/>
+      <c r="F102" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G102" s="46" t="s">
+        <v>61</v>
+      </c>
+      <c r="H102" s="19"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103" s="60"/>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
-      <c r="D103" s="28" t="s">
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="F103" s="1"/>
+      <c r="G103" s="45" t="s">
         <v>97</v>
-      </c>
-      <c r="E103" s="1"/>
-      <c r="F103" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="G103" s="46" t="s">
-        <v>99</v>
       </c>
       <c r="H103" s="19"/>
     </row>
@@ -8781,133 +8725,133 @@
       <c r="A104" s="60"/>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
-      <c r="D104" s="2" t="s">
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1"/>
+      <c r="G104" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E104" s="1"/>
-      <c r="F104" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G104" s="46"/>
       <c r="H104" s="19"/>
     </row>
     <row r="105" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="59"/>
+      <c r="A105" s="58"/>
       <c r="B105" s="17"/>
       <c r="C105" s="17"/>
       <c r="D105" s="17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E105" s="17"/>
       <c r="F105" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="G105" s="48"/>
+        <v>110</v>
+      </c>
+      <c r="G105" s="17" t="s">
+        <v>115</v>
+      </c>
       <c r="H105" s="18"/>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A106" s="58" t="s">
-        <v>123</v>
+      <c r="A106" s="57" t="s">
+        <v>121</v>
       </c>
       <c r="B106" s="13"/>
       <c r="C106" s="14"/>
-      <c r="D106" s="32" t="s">
+      <c r="D106" s="31" t="s">
         <v>12</v>
       </c>
       <c r="E106" s="14"/>
       <c r="F106" s="14"/>
-      <c r="G106" s="32" t="s">
-        <v>68</v>
+      <c r="G106" s="31" t="s">
+        <v>66</v>
       </c>
       <c r="H106" s="15"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A107" s="60"/>
+      <c r="A107" s="59"/>
       <c r="B107" s="1"/>
       <c r="C107" s="1"/>
-      <c r="D107" s="33" t="s">
-        <v>49</v>
+      <c r="D107" s="32" t="s">
+        <v>47</v>
       </c>
       <c r="E107" s="1"/>
       <c r="F107" s="1"/>
-      <c r="G107" s="33" t="s">
-        <v>124</v>
+      <c r="G107" s="32" t="s">
+        <v>122</v>
       </c>
       <c r="H107" s="19"/>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A108" s="60"/>
+      <c r="A108" s="59"/>
       <c r="B108" s="1"/>
       <c r="C108" s="1"/>
-      <c r="D108" s="33"/>
+      <c r="D108" s="32"/>
       <c r="E108" s="1"/>
       <c r="F108" s="1"/>
-      <c r="G108" s="34" t="s">
+      <c r="G108" s="33" t="s">
         <v>12</v>
       </c>
       <c r="H108" s="19"/>
       <c r="K108" s="23"/>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A109" s="60"/>
+      <c r="A109" s="59"/>
       <c r="B109" s="1"/>
       <c r="C109" s="1"/>
-      <c r="D109" s="33"/>
+      <c r="D109" s="32"/>
       <c r="E109" s="1"/>
       <c r="F109" s="1"/>
-      <c r="G109" s="33" t="s">
-        <v>70</v>
+      <c r="G109" s="32" t="s">
+        <v>68</v>
       </c>
       <c r="H109" s="19"/>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A110" s="60"/>
+      <c r="A110" s="59"/>
       <c r="B110" s="1"/>
       <c r="C110" s="1"/>
-      <c r="D110" s="33"/>
+      <c r="D110" s="32"/>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
-      <c r="G110" s="47" t="s">
-        <v>63</v>
+      <c r="G110" s="46" t="s">
+        <v>61</v>
       </c>
       <c r="H110" s="19"/>
     </row>
     <row r="111" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="59"/>
+      <c r="A111" s="58"/>
       <c r="B111" s="17"/>
       <c r="C111" s="17"/>
-      <c r="D111" s="41"/>
+      <c r="D111" s="40"/>
       <c r="E111" s="17"/>
       <c r="F111" s="17"/>
-      <c r="G111" s="48" t="s">
-        <v>125</v>
+      <c r="G111" s="47" t="s">
+        <v>123</v>
       </c>
       <c r="H111" s="18"/>
     </row>
     <row r="112" spans="1:11" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B112" s="62"/>
-      <c r="C112" s="62"/>
-      <c r="D112" s="62"/>
-      <c r="E112" s="62"/>
-      <c r="F112" s="62"/>
-      <c r="G112" s="62"/>
-      <c r="H112" s="62"/>
+      <c r="B112" s="61"/>
+      <c r="C112" s="61"/>
+      <c r="D112" s="61"/>
+      <c r="E112" s="61"/>
+      <c r="F112" s="61"/>
+      <c r="G112" s="61"/>
+      <c r="H112" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="B112:H112"/>
-    <mergeCell ref="B101:H101"/>
+    <mergeCell ref="B99:H99"/>
     <mergeCell ref="B45:H45"/>
     <mergeCell ref="B56:H56"/>
-    <mergeCell ref="A93:A96"/>
-    <mergeCell ref="A97:A100"/>
-    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="A91:A94"/>
+    <mergeCell ref="A95:A98"/>
+    <mergeCell ref="A100:A105"/>
     <mergeCell ref="A106:A111"/>
     <mergeCell ref="A67:A68"/>
     <mergeCell ref="A69:A72"/>
     <mergeCell ref="A73:A76"/>
     <mergeCell ref="A77:A86"/>
-    <mergeCell ref="A87:A92"/>
+    <mergeCell ref="A87:A90"/>
     <mergeCell ref="A46:A47"/>
     <mergeCell ref="A48:A51"/>
     <mergeCell ref="A52:A55"/>
@@ -8943,36 +8887,36 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="69" t="s">
-        <v>126</v>
-      </c>
-      <c r="C4" s="69"/>
-      <c r="D4" s="69"/>
-      <c r="E4" s="69"/>
+      <c r="B4" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="68"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="70" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="70"/>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
+      <c r="B5" s="69" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="69"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -9028,7 +8972,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7">
         <v>0</v>
@@ -9045,7 +8989,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B11" s="7">
         <v>0</v>
@@ -9062,7 +9006,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B12" s="7">
         <v>0</v>
@@ -9079,7 +9023,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B13" s="7">
         <v>0</v>
@@ -9096,7 +9040,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B14" s="7">
         <v>0</v>
@@ -9113,7 +9057,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B15" s="7">
         <v>0</v>
@@ -9130,7 +9074,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B16" s="7">
         <v>0</v>
@@ -9147,7 +9091,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B17" s="7">
         <v>0</v>
@@ -9164,7 +9108,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B18" s="7">
         <v>0</v>
@@ -9181,7 +9125,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B19" s="7">
         <v>0</v>
@@ -9198,7 +9142,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B20" s="7">
         <v>0</v>
@@ -9215,7 +9159,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B21" s="7">
         <v>0</v>
@@ -9232,7 +9176,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B22" s="7">
         <v>0</v>
@@ -9249,7 +9193,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B23" s="7">
         <v>0</v>
@@ -9266,7 +9210,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B24" s="7">
         <v>0</v>
@@ -9283,7 +9227,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B25" s="7">
         <v>0</v>
@@ -9300,7 +9244,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" s="7">
         <v>0</v>
@@ -9317,7 +9261,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B27" s="7">
         <v>0</v>
@@ -9334,7 +9278,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B28" s="7">
         <v>0</v>
@@ -9351,7 +9295,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B29" s="7">
         <v>0</v>
@@ -9368,7 +9312,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B30" s="7">
         <v>0</v>
@@ -9385,7 +9329,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B31" s="7">
         <v>0</v>
@@ -9402,7 +9346,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B32" s="7">
         <v>0</v>
@@ -9419,7 +9363,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B33" s="7">
         <v>0</v>
@@ -9436,7 +9380,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B34" s="7">
         <v>0</v>
@@ -9486,40 +9430,40 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>